<commit_message>
Zadania: autorska agenda warsztatow analizy KP (kolejnosc wg zaleznosci danych w enova365, pracownicy wzorcowi, pokaz na danych klienta); generator rozdzielony na dwa warianty
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdibRG4Pgk3Z3PYuVYVwnZ
</commit_message>
<xml_diff>
--- a/Zadania/Agenda warsztatów analizy KP/Agenda warsztatów analizy KP.xlsx
+++ b/Zadania/Agenda warsztatów analizy KP/Agenda warsztatów analizy KP.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
-    <t>Agenda warsztatów analizy przedwdrożeniowej – Kadry, Płace, Czas pracy (enova365)</t>
+    <t>Agenda warsztatów analizy przedwdrożeniowej – Kadry, Płace, Czas pracy (enova365) – korekta agendy wyjściowej</t>
   </si>
   <si>
     <t>Źródło: Twoja agenda | Umowa – brak w agendzie (pomarańczowe) | Dodane (metodyka, zielone). „s. N” = strona instrukcji „Kadry Płace i HR”, (P) = licencja Platynowa, (Z) = Złota. Odwołania rozdz./KAD-/CP-/PL- – dokument analizy w Analiza/.</t>
@@ -3014,7 +3014,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.710938" customWidth="1"/>
+    <col min="2" max="2" width="28.710938" customWidth="1"/>
     <col min="3" max="3" width="70.71094" customWidth="1"/>
     <col min="4" max="4" width="80.71094" customWidth="1"/>
   </cols>

</xml_diff>